<commit_message>
Development is in progress
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-con2\Documents\UiPath\AMP14_00_LiberarCalculoCoste\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BF46CC-7800-4C79-A9DD-1FDC89055229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC08C2C-4489-4330-865F-62FE950C529E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="75">
   <si>
     <t>Name</t>
   </si>
@@ -221,39 +221,55 @@
     <t>InitialInpuPath</t>
   </si>
   <si>
-    <t>LCCoste_InitialInpuPath</t>
-  </si>
-  <si>
     <t>Ruta del insumo inicial incluido el nombre del archivo</t>
   </si>
   <si>
     <t>InputSheetName</t>
   </si>
   <si>
-    <t>LCCoste_InputSheetName</t>
-  </si>
-  <si>
     <t>Nombre de la hoja por procesar del insumo inicial</t>
   </si>
   <si>
-    <t>Valores para iterar para la variante de costo y control ttraspaso</t>
-  </si>
-  <si>
-    <t>LCCoste_VarianteCostoTraspaso</t>
-  </si>
-  <si>
-    <t>VarianteCostoTraspaso</t>
+    <t>ISR_SAPVariantes</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Nombres de variantes en SAP</t>
+  </si>
+  <si>
+    <t>SAPVariantes</t>
+  </si>
+  <si>
+    <t>ISR_SAPDisposicion</t>
+  </si>
+  <si>
+    <t>SAPDisposicion</t>
+  </si>
+  <si>
+    <t>Nombres de disposicion en SAP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -342,13 +358,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2841,7 +2858,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z984"/>
+  <dimension ref="A1:Z983"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -2960,45 +2977,58 @@
       <c r="A7" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>64</v>
+      <c r="B7" s="11" t="s">
+        <v>68</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>67</v>
+        <v>65</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>69</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>70</v>
+      <c r="B9" s="11" t="s">
+        <v>67</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>69</v>
+      <c r="D9" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3192,7 +3222,7 @@
     <row r="201" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="202" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="203" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="204" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3972,7 +4002,6 @@
     <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>